<commit_message>
tercer commit, mejora de articulos y plantilla de excel
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_relevo.xlsx
+++ b/plantillas/plantilla_relevo.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\rosamudio\Desktop\Proy_Scan_Patrimonio\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3164AA3C-5E2A-4A3D-BCC1-B07682F59E27}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D86097F-2BE0-416D-9C45-91A8C4C157CE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{C6269841-EB62-4CEF-B92A-5D26EE27050D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$I$23</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>FECHA:</t>
   </si>
@@ -64,15 +67,64 @@
   </si>
   <si>
     <t>OBSERVACIONES</t>
+  </si>
+  <si>
+    <t>RESPONSABLE:</t>
+  </si>
+  <si>
+    <t>SUBRESPONSABLE:</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ACTA DE RELEVAMIENTO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Coordinación de Patrimonio y Suministros</t>
+    </r>
+  </si>
+  <si>
+    <t>SECTOR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -125,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -135,6 +187,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -156,133 +215,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>3659</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>56532</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Imagen 9">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B63E90B-F68D-4CC0-95DC-425B3265A88E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="3659"/>
-          <a:ext cx="6686550" cy="605323"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>704850</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Rectángulo: esquinas redondeadas 10">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE557A7C-B809-4A5C-A52D-149B7364A1FB}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2362200" y="0"/>
-          <a:ext cx="3314700" cy="552450"/>
-        </a:xfrm>
-        <a:prstGeom prst="roundRect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="50000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-AR" sz="1100"/>
-            <a:t>ACTA</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-AR" sz="1100" baseline="0"/>
-            <a:t> DE RELEVAMIENTO</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-AR" sz="1100" baseline="0"/>
-            <a:t>Coordinación de Patrimonio y Suministros</a:t>
-          </a:r>
-          <a:endParaRPr lang="es-AR" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -582,45 +514,82 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{978991BD-5560-402D-9B63-8BC0815204ED}">
-  <dimension ref="A5:H13"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="2" max="2" width="14.08984375" customWidth="1"/>
+    <col min="1" max="1" width="6.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" customWidth="1"/>
     <col min="3" max="3" width="13.6328125" customWidth="1"/>
+    <col min="4" max="4" width="18.36328125" customWidth="1"/>
     <col min="8" max="8" width="14.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="G5" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C8" s="3"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E9" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="3"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>5</v>
       </c>
@@ -645,10 +614,22 @@
       <c r="H13" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="I13" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I14" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:G3"/>
+  </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" scale="90" fitToHeight="0" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;G</oddHeader>
+  </headerFooter>
+  <legacyDrawingHF r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
actualizacion del modo oscuro, agregaod de etiquetas para planilla_relevo, ordenamiento, mejora visual
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_relevo.xlsx
+++ b/plantillas/plantilla_relevo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\rosamudio\Desktop\Proy_Scan_Patrimonio\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D86097F-2BE0-416D-9C45-91A8C4C157CE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6833E23-0BE5-4147-A6E0-A7EC0ACD22F0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{C6269841-EB62-4CEF-B92A-5D26EE27050D}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>FECHA:</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>SECTOR</t>
+  </si>
+  <si>
+    <t>TELEFONO:</t>
   </si>
 </sst>
 </file>
@@ -582,12 +585,18 @@
         <v>3</v>
       </c>
       <c r="C10" s="4"/>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B11" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="3"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
@@ -626,7 +635,7 @@
     <mergeCell ref="C1:G3"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="90" fitToHeight="0" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="90" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;G</oddHeader>
   </headerFooter>

</xml_diff>